<commit_message>
feat: Add dropdown validation for statusDetail column
</commit_message>
<xml_diff>
--- a/07-partner-accounts/Leta_Application_Tracker.xlsx
+++ b/07-partner-accounts/Leta_Application_Tracker.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="79">
   <si>
     <t>Platform</t>
   </si>
@@ -174,9 +174,6 @@
   </si>
   <si>
     <t>Not Started</t>
-  </si>
-  <si>
-    <t>In Progress</t>
   </si>
   <si>
     <t>federal subcontract baseline</t>
@@ -709,7 +706,7 @@
         <v>52</v>
       </c>
       <c r="E2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -726,7 +723,7 @@
         <v>52</v>
       </c>
       <c r="E3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -743,7 +740,7 @@
         <v>52</v>
       </c>
       <c r="E4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -760,7 +757,7 @@
         <v>52</v>
       </c>
       <c r="E5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -777,7 +774,7 @@
         <v>52</v>
       </c>
       <c r="E6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -794,7 +791,7 @@
         <v>52</v>
       </c>
       <c r="E7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -811,7 +808,7 @@
         <v>52</v>
       </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -828,7 +825,7 @@
         <v>52</v>
       </c>
       <c r="E9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -842,13 +839,13 @@
         <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -865,7 +862,7 @@
         <v>52</v>
       </c>
       <c r="E11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -882,7 +879,7 @@
         <v>52</v>
       </c>
       <c r="E12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -899,7 +896,7 @@
         <v>52</v>
       </c>
       <c r="E13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -916,7 +913,7 @@
         <v>52</v>
       </c>
       <c r="E14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -933,7 +930,7 @@
         <v>52</v>
       </c>
       <c r="E15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -950,7 +947,7 @@
         <v>52</v>
       </c>
       <c r="E16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -967,7 +964,7 @@
         <v>52</v>
       </c>
       <c r="E17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -984,7 +981,7 @@
         <v>52</v>
       </c>
       <c r="E18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1001,7 +998,7 @@
         <v>52</v>
       </c>
       <c r="E19" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -1018,7 +1015,7 @@
         <v>52</v>
       </c>
       <c r="E20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -1035,13 +1032,13 @@
         <v>52</v>
       </c>
       <c r="E21" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D100">
-      <formula1>"Not Started,In Progress,Submitted,Under Review,Approved,Rejected"</formula1>
+      <formula1>"Not Started,Submitted,Under Review,Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -1081,15 +1078,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1103,10 +1100,10 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
       <c r="B5">
-        <f>COUNTIF(Tracker!D:D, "In Progress")</f>
+        <f>COUNTIF(Tracker!D:D, "Submitted")</f>
         <v>0</v>
       </c>
     </row>
@@ -1115,7 +1112,7 @@
         <v>75</v>
       </c>
       <c r="B6">
-        <f>COUNTIF(Tracker!D:D, "Submitted")</f>
+        <f>COUNTIF(Tracker!D:D, "Under Review")</f>
         <v>0</v>
       </c>
     </row>
@@ -1124,7 +1121,7 @@
         <v>76</v>
       </c>
       <c r="B7">
-        <f>COUNTIF(Tracker!D:D, "Under Review")</f>
+        <f>COUNTIF(Tracker!D:D, "Approved")</f>
         <v>0</v>
       </c>
     </row>
@@ -1133,22 +1130,13 @@
         <v>77</v>
       </c>
       <c r="B8">
-        <f>COUNTIF(Tracker!D:D, "Approved")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" t="s">
-        <v>78</v>
-      </c>
-      <c r="B9">
         <f>COUNTIF(Tracker!D:D, "Rejected")</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B10" s="5">
         <f>COUNTA(Tracker!A:A)-1</f>

</xml_diff>